<commit_message>
Aplica o novo logo da Lócus no site, painel e planilha do cliente
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CQ2ucupGpT3694nT6vbTKk
</commit_message>
<xml_diff>
--- a/locus/painel/Planilha_Lancamentos_Locus.xlsx
+++ b/locus/painel/Planilha_Lancamentos_Locus.xlsx
@@ -30,7 +30,7 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="102" uniqueCount="65">
   <si>
-    <t xml:space="preserve">LÓCUS  ·  DIAGNÓSTICO FINANCEIRO</t>
+    <t xml:space="preserve">DIAGNÓSTICO FINANCEIRO</t>
   </si>
   <si>
     <t xml:space="preserve">Contabilidade guiada por dados · Pompéu – MG</t>
@@ -93,7 +93,7 @@
     <t xml:space="preserve">paulosergio4.github.io/meus-projetos/locus</t>
   </si>
   <si>
-    <t xml:space="preserve">LÓCUS  ·  LANÇAMENTOS</t>
+    <t xml:space="preserve">LANÇAMENTOS</t>
   </si>
   <si>
     <t xml:space="preserve">Uma linha por movimento. Os campos com lista abrem ao clicar na célula.</t>
@@ -150,7 +150,7 @@
     <t xml:space="preserve">Energia, água e internet</t>
   </si>
   <si>
-    <t xml:space="preserve">LÓCUS  ·  RESUMO</t>
+    <t xml:space="preserve">RESUMO</t>
   </si>
   <si>
     <t xml:space="preserve">Calculado automaticamente a partir dos lançamentos.</t>
@@ -994,6 +994,132 @@
 </styleSheet>
 </file>
 
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>1695240</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>475920</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="0" name="Image 1" descr="Picture"/>
+        <xdr:cNvPicPr/>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip r:embed="rId1"/>
+        <a:stretch/>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="5991120" y="152280"/>
+          <a:ext cx="1695240" cy="475920"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln w="0">
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>1695240</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>475920</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="1" name="Image 1" descr="Picture"/>
+        <xdr:cNvPicPr/>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip r:embed="rId1"/>
+        <a:stretch/>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="8035200" y="152280"/>
+          <a:ext cx="1695240" cy="475920"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln w="0">
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>214920</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>475920</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Image 1" descr="Picture"/>
+        <xdr:cNvPicPr/>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip r:embed="rId1"/>
+        <a:stretch/>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="8669520" y="152280"/>
+          <a:ext cx="1695240" cy="475920"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln w="0">
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="tbLancamentos" displayName="tbLancamentos" ref="B7:G507" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <autoFilter ref="B7:G507"/>
@@ -7751,6 +7877,7 @@
     <oddHeader/>
     <oddFooter/>
   </headerFooter>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -45301,8 +45428,9 @@
     <oddHeader/>
     <oddFooter/>
   </headerFooter>
+  <drawing r:id="rId1"/>
   <tableParts>
-    <tablePart r:id="rId1"/>
+    <tablePart r:id="rId2"/>
   </tableParts>
 </worksheet>
 </file>
@@ -51994,7 +52122,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{7C15EFC1-997A-46DB-A476-8EAADCC17D12}</x14:id>
+          <x14:id>{178A3080-9389-4C76-B3BB-21EE623966D5}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -52006,11 +52134,12 @@
     <oddHeader/>
     <oddFooter/>
   </headerFooter>
+  <drawing r:id="rId1"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{7C15EFC1-997A-46DB-A476-8EAADCC17D12}">
+          <x14:cfRule type="dataBar" id="{178A3080-9389-4C76-B3BB-21EE623966D5}">
             <x14:dataBar minLength="10" maxLength="90" axisPosition="none" gradient="true">
               <x14:cfvo type="min"/>
               <x14:cfvo type="max"/>

</xml_diff>